<commit_message>
Aligning Github and Zenodo
Checking that the data are actually the same update between Zenodo and Github
</commit_message>
<xml_diff>
--- a/3_CGE/Game_theory_2024/0_External_data/Original_EV.xlsx
+++ b/3_CGE/Game_theory_2024/0_External_data/Original_EV.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\runGTAP375\Game_theory_2024\0_External_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9D1E6F7-8938-49CA-B8EF-C2F3315CD8A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B19B2859-CE62-4A1C-A086-072C3C9A4862}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41250" yWindow="10875" windowWidth="14400" windowHeight="7365" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="624" yWindow="1428" windowWidth="19176" windowHeight="10176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EV" sheetId="1" r:id="rId1"/>
@@ -560,9 +560,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -600,7 +600,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -706,7 +706,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -848,7 +848,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -856,194 +856,219 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A37"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:A42"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A38" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A39" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A40" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A41" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A42" s="1">
         <v>0</v>
       </c>
     </row>

</xml_diff>